<commit_message>
Remove obsolete mercury test data file; update UltraArm_P1 test data file; add new test case for setting digital IO output with normal and exception scenarios.
</commit_message>
<xml_diff>
--- a/test_data/UltraArm_P1.xlsx
+++ b/test_data/UltraArm_P1.xlsx
@@ -4,30 +4,31 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="10500" firstSheet="3" activeTab="3"/>
+    <workbookView windowWidth="22188" windowHeight="10500" firstSheet="17" activeTab="21"/>
   </bookViews>
   <sheets>
     <sheet name="get_system_version" sheetId="1" r:id="rId1"/>
-    <sheet name="get_modify_version" sheetId="3" r:id="rId2"/>
-    <sheet name="set_angles" sheetId="19" r:id="rId3"/>
-    <sheet name="set_angle" sheetId="21" r:id="rId4"/>
-    <sheet name="get_angles_info" sheetId="18" r:id="rId5"/>
-    <sheet name="set_coords" sheetId="23" r:id="rId6"/>
-    <sheet name="set_coord" sheetId="24" r:id="rId7"/>
-    <sheet name="get_error_information" sheetId="11" r:id="rId8"/>
-    <sheet name="get_coords_info" sheetId="22" r:id="rId9"/>
-    <sheet name="set_jog_angle" sheetId="31" r:id="rId10"/>
-    <sheet name="stop" sheetId="28" r:id="rId11"/>
-    <sheet name="is_moving" sheetId="30" r:id="rId12"/>
-    <sheet name="jog_rpy" sheetId="32" r:id="rId13"/>
-    <sheet name="set_jog_coord" sheetId="33" r:id="rId14"/>
-    <sheet name="jog_increment_angle" sheetId="34" r:id="rId15"/>
-    <sheet name="jog_increment_coord" sheetId="35" r:id="rId16"/>
-    <sheet name="set_zero_calibration" sheetId="45" r:id="rId17"/>
-    <sheet name="set_base_io_output" sheetId="52" r:id="rId18"/>
-    <sheet name="set_joint_enable" sheetId="53" r:id="rId19"/>
-    <sheet name="set_joint_release" sheetId="54" r:id="rId20"/>
-    <sheet name="Sheet3" sheetId="55" r:id="rId21"/>
+    <sheet name="get_modify_version" sheetId="2" r:id="rId2"/>
+    <sheet name="set_angles" sheetId="3" r:id="rId3"/>
+    <sheet name="set_angle" sheetId="4" r:id="rId4"/>
+    <sheet name="get_angles_info" sheetId="5" r:id="rId5"/>
+    <sheet name="set_coords" sheetId="6" r:id="rId6"/>
+    <sheet name="set_coord" sheetId="7" r:id="rId7"/>
+    <sheet name="get_error_information" sheetId="8" r:id="rId8"/>
+    <sheet name="get_coords_info" sheetId="9" r:id="rId9"/>
+    <sheet name="set_jog_angle" sheetId="10" r:id="rId10"/>
+    <sheet name="stop" sheetId="11" r:id="rId11"/>
+    <sheet name="is_moving" sheetId="12" r:id="rId12"/>
+    <sheet name="jog_rpy" sheetId="13" r:id="rId13"/>
+    <sheet name="set_jog_coord" sheetId="14" r:id="rId14"/>
+    <sheet name="jog_increment_angle" sheetId="15" r:id="rId15"/>
+    <sheet name="jog_increment_coord" sheetId="16" r:id="rId16"/>
+    <sheet name="set_zero_calibration" sheetId="17" r:id="rId17"/>
+    <sheet name="set_base_io_output" sheetId="18" r:id="rId18"/>
+    <sheet name="set_joint_enable" sheetId="19" r:id="rId19"/>
+    <sheet name="set_joint_release" sheetId="20" r:id="rId20"/>
+    <sheet name="Sheet3" sheetId="21" r:id="rId21"/>
+    <sheet name="set_digital_io_output" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="259">
   <si>
     <t>ID</t>
   </si>
@@ -803,6 +804,27 @@
   </si>
   <si>
     <t>set_joint_release</t>
+  </si>
+  <si>
+    <t>引脚1高电平</t>
+  </si>
+  <si>
+    <t>set_digital_io_output</t>
+  </si>
+  <si>
+    <t>引脚1低电平</t>
+  </si>
+  <si>
+    <t>引脚2高电平</t>
+  </si>
+  <si>
+    <t>引脚2低电平</t>
+  </si>
+  <si>
+    <t>引脚号超限</t>
+  </si>
+  <si>
+    <t>状态非法</t>
   </si>
 </sst>
 </file>
@@ -1419,7 +1441,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1429,15 +1451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1755,7 +1769,7 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="2" max="6" width="18" customWidth="1"/>
+    <col min="2" max="6" width="18" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1774,25 +1788,25 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="28.8" spans="1:6">
+    <row r="2" ht="28.8" customHeight="1" spans="1:6">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="6">
-        <v>1</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1817,7 +1831,7 @@
     <col min="6" max="6" width="28.5" style="2" customWidth="1"/>
     <col min="7" max="8" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="9" max="9" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="1"/>
+    <col min="10" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:9">
@@ -1907,7 +1921,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="4" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1936,7 +1950,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="5" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1965,7 +1979,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="6" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1994,7 +2008,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="7" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2023,7 +2037,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="8" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2052,7 +2066,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="28.8" spans="1:9">
+    <row r="9" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:9">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -2254,13 +2268,13 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="28.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2369,13 +2383,13 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.6296296296296" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2450,7 +2464,7 @@
     <col min="5" max="5" width="21.6296296296296" style="2" customWidth="1"/>
     <col min="6" max="7" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -2531,7 +2545,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="4" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2557,7 +2571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="5" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2583,7 +2597,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="6" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2609,7 +2623,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="7" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2635,7 +2649,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="8" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A8" s="2">
         <v>13</v>
       </c>
@@ -2661,7 +2675,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="9" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A9" s="2">
         <v>14</v>
       </c>
@@ -2687,7 +2701,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="10" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A10" s="2">
         <v>15</v>
       </c>
@@ -2713,7 +2727,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="11" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A11" s="2">
         <v>16</v>
       </c>
@@ -2739,7 +2753,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="12" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A12" s="2">
         <v>17</v>
       </c>
@@ -2765,7 +2779,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="13" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A13" s="2">
         <v>18</v>
       </c>
@@ -2954,7 +2968,7 @@
     <col min="5" max="5" width="21.6296296296296" style="2" customWidth="1"/>
     <col min="6" max="7" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -3035,7 +3049,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="4" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -3061,7 +3075,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="5" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -3087,7 +3101,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="6" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -3113,7 +3127,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="7" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -3139,7 +3153,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="8" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -3165,7 +3179,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="9" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3191,7 +3205,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="10" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3217,7 +3231,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="11" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3243,7 +3257,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="12" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3269,7 +3283,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="13" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3295,7 +3309,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="14" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3321,7 +3335,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="15" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3347,7 +3361,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="16" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3373,7 +3387,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="17" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3399,7 +3413,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="18" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3425,7 +3439,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="19" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3451,7 +3465,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="20" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3477,7 +3491,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="21" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3503,7 +3517,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="22" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3529,7 +3543,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="23" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3555,7 +3569,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="24" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3581,7 +3595,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="25" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3770,7 +3784,7 @@
     <col min="5" max="5" width="21.6296296296296" style="2" customWidth="1"/>
     <col min="6" max="7" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -3851,7 +3865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="4" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -3877,7 +3891,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="5" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -3903,7 +3917,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="6" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -3929,7 +3943,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="7" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -3955,7 +3969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="8" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -3981,7 +3995,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="9" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4007,7 +4021,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="10" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4033,7 +4047,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="11" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -4059,7 +4073,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="12" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -4085,7 +4099,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="13" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -4111,7 +4125,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="14" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4137,7 +4151,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="15" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -4163,7 +4177,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="16" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -4189,7 +4203,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="17" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -4215,7 +4229,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="18" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4241,7 +4255,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="19" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -4267,7 +4281,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="20" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4293,7 +4307,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="21" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -4319,7 +4333,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="22" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -4345,7 +4359,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="23" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -4371,7 +4385,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="24" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -4397,7 +4411,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="43.2" spans="1:8">
+    <row r="25" s="1" customFormat="1" ht="43.2" customHeight="1" spans="1:8">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -4423,7 +4437,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="26" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -4447,7 +4461,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="27" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -4471,7 +4485,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="28" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -4495,7 +4509,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="29" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -4519,7 +4533,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="30" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -4543,7 +4557,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="31" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -4586,7 +4600,7 @@
     <col min="5" max="5" width="21.6296296296296" style="2" customWidth="1"/>
     <col min="6" max="7" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -4667,7 +4681,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="4" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -4719,7 +4733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="6" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -4745,7 +4759,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="7" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -4771,7 +4785,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="8" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4797,7 +4811,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="9" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4823,7 +4837,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="10" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4849,7 +4863,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="11" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -4875,7 +4889,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="12" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -4901,7 +4915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="13" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -4927,7 +4941,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="14" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4953,7 +4967,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="15" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -4979,7 +4993,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="16" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -5005,7 +5019,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="17" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -5031,7 +5045,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="18" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -5057,7 +5071,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="19" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -5083,7 +5097,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="20" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -5109,7 +5123,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="21" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -5135,7 +5149,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="22" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -5161,7 +5175,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="23" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -5187,7 +5201,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="24" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -5213,7 +5227,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="25" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -5239,7 +5253,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="26" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -5263,7 +5277,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="27" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -5287,7 +5301,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="28" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -5311,7 +5325,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="29" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -5335,7 +5349,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="30" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -5359,7 +5373,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="31" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -5398,10 +5412,10 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="28.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -5424,7 +5438,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="2" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
         <v>225</v>
@@ -5482,7 +5496,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="5" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -5502,7 +5516,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="6" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -5522,7 +5536,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="7" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -5539,7 +5553,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="8" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -5572,7 +5586,7 @@
     <col min="2" max="3" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="4" max="6" width="28.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="8" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -6245,13 +6259,13 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.6296296296296" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6300,7 +6314,7 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="2" max="6" width="18" customWidth="1"/>
+    <col min="2" max="6" width="18" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6319,25 +6333,25 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="28.8" spans="1:6">
+    <row r="2" ht="28.8" customHeight="1" spans="1:6">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="5">
-        <v>0</v>
-      </c>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -6357,13 +6371,13 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.8796296296296" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.6296296296296" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6417,6 +6431,183 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="6"/>
+  <cols>
+    <col min="2" max="2" width="16.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="21.5555555555556" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>231</v>
+      </c>
+      <c r="E1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C3" t="s">
+        <v>253</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4" t="s">
+        <v>253</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>256</v>
+      </c>
+      <c r="C5" t="s">
+        <v>253</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D6">
+        <v>99</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C7" t="s">
+        <v>253</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
@@ -6428,7 +6619,7 @@
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
     <col min="4" max="4" width="28.5" style="1" customWidth="1"/>
     <col min="5" max="7" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="8" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -6500,7 +6691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" ht="28.8" spans="1:7">
+    <row r="4" ht="28.8" customHeight="1" spans="1:7">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -6523,7 +6714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="28.8" spans="1:7">
+    <row r="5" ht="28.8" customHeight="1" spans="1:7">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -6546,7 +6737,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="28.8" spans="1:7">
+    <row r="6" ht="28.8" customHeight="1" spans="1:7">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -6569,7 +6760,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" ht="28.8" spans="1:7">
+    <row r="7" ht="28.8" customHeight="1" spans="1:7">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -6592,7 +6783,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" ht="28.8" spans="1:7">
+    <row r="8" ht="28.8" customHeight="1" spans="1:7">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -6615,7 +6806,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" ht="28.8" spans="1:7">
+    <row r="9" ht="28.8" customHeight="1" spans="1:7">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -6638,7 +6829,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" ht="28.8" spans="1:7">
+    <row r="10" ht="28.8" customHeight="1" spans="1:7">
       <c r="A10" s="2">
         <v>25</v>
       </c>
@@ -6655,7 +6846,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" ht="28.8" spans="1:7">
+    <row r="11" ht="28.8" customHeight="1" spans="1:7">
       <c r="A11" s="2">
         <v>26</v>
       </c>
@@ -6672,7 +6863,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" ht="28.8" spans="1:7">
+    <row r="12" ht="28.8" customHeight="1" spans="1:7">
       <c r="A12" s="2">
         <v>27</v>
       </c>
@@ -6689,7 +6880,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" ht="28.8" spans="1:7">
+    <row r="13" ht="28.8" customHeight="1" spans="1:7">
       <c r="A13" s="2">
         <v>28</v>
       </c>
@@ -6706,7 +6897,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" ht="28.8" spans="1:7">
+    <row r="14" ht="28.8" customHeight="1" spans="1:7">
       <c r="A14" s="2">
         <v>29</v>
       </c>
@@ -6723,7 +6914,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" ht="28.8" spans="1:7">
+    <row r="15" ht="28.8" customHeight="1" spans="1:7">
       <c r="A15" s="2">
         <v>30</v>
       </c>
@@ -6740,7 +6931,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" ht="28.8" spans="1:7">
+    <row r="16" ht="28.8" customHeight="1" spans="1:7">
       <c r="A16" s="2">
         <v>31</v>
       </c>
@@ -6757,7 +6948,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" ht="28.8" spans="1:7">
+    <row r="17" ht="28.8" customHeight="1" spans="1:7">
       <c r="A17" s="2">
         <v>32</v>
       </c>
@@ -6774,7 +6965,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" ht="28.8" spans="1:7">
+    <row r="18" ht="28.8" customHeight="1" spans="1:7">
       <c r="A18" s="2">
         <v>37</v>
       </c>
@@ -6794,7 +6985,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" ht="28.8" spans="1:7">
+    <row r="19" ht="28.8" customHeight="1" spans="1:7">
       <c r="A19" s="2">
         <v>38</v>
       </c>
@@ -6831,7 +7022,7 @@
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
     <col min="4" max="5" width="28.5" style="1" customWidth="1"/>
     <col min="6" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -6912,7 +7103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="4" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -6938,7 +7129,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="5" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -6964,7 +7155,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="6" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -6990,7 +7181,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="7" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -7016,7 +7207,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="8" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -7042,7 +7233,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="9" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -7068,7 +7259,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="10" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A10" s="2">
         <v>25</v>
       </c>
@@ -7091,7 +7282,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="11" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A11" s="2">
         <v>26</v>
       </c>
@@ -7114,7 +7305,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="12" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A12" s="2">
         <v>27</v>
       </c>
@@ -7137,7 +7328,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="13" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A13" s="2">
         <v>28</v>
       </c>
@@ -7160,7 +7351,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="14" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A14" s="2">
         <v>29</v>
       </c>
@@ -7183,7 +7374,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="15" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A15" s="2">
         <v>30</v>
       </c>
@@ -7206,7 +7397,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="16" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A16" s="2">
         <v>31</v>
       </c>
@@ -7229,7 +7420,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="17" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A17" s="2">
         <v>32</v>
       </c>
@@ -7313,13 +7504,13 @@
     <col min="1" max="1" width="13.2222222222222" style="2" customWidth="1"/>
     <col min="2" max="2" width="16.1111111111111" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1"/>
+    <col min="4" max="4" width="9" style="1" customWidth="1"/>
     <col min="5" max="5" width="28.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:6">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7390,7 +7581,7 @@
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
     <col min="4" max="4" width="48.25" style="1" customWidth="1"/>
     <col min="5" max="7" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="8" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:14">
@@ -7554,7 +7745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="8" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -7577,7 +7768,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="9" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -7600,7 +7791,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="10" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A10" s="2">
         <v>25</v>
       </c>
@@ -7620,7 +7811,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="11" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A11" s="2">
         <v>26</v>
       </c>
@@ -7637,7 +7828,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="12" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A12" s="2">
         <v>27</v>
       </c>
@@ -7654,7 +7845,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="13" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A13" s="2">
         <v>28</v>
       </c>
@@ -7671,7 +7862,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="14" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A14" s="2">
         <v>29</v>
       </c>
@@ -7688,7 +7879,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="15" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A15" s="2">
         <v>30</v>
       </c>
@@ -7705,7 +7896,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="28.8" spans="1:14">
+    <row r="16" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:14">
       <c r="A16" s="2">
         <v>31</v>
       </c>
@@ -7725,7 +7916,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="28.8" spans="1:7">
+    <row r="17" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:7">
       <c r="A17" s="2">
         <v>32</v>
       </c>
@@ -7764,7 +7955,7 @@
     <col min="5" max="5" width="19.6296296296296" style="2" customWidth="1"/>
     <col min="6" max="7" width="13.5555555555556" style="2" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:8">
@@ -8209,12 +8400,12 @@
     <col min="2" max="2" width="16.1111111111111" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" style="1" customWidth="1"/>
     <col min="4" max="4" width="21.6296296296296" style="1" customWidth="1"/>
-    <col min="5" max="7" width="9" style="1"/>
+    <col min="5" max="7" width="9" style="1" customWidth="1"/>
     <col min="8" max="8" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:8">
+    <row r="1" s="1" customFormat="1" ht="28.8" customHeight="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8283,7 +8474,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" ht="43.2" spans="1:8">
+    <row r="4" ht="43.2" customHeight="1" spans="1:8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -8309,7 +8500,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" ht="43.2" spans="1:8">
+    <row r="5" ht="43.2" customHeight="1" spans="1:8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -8353,7 +8544,7 @@
     <col min="4" max="4" width="20.3796296296296" style="1" customWidth="1"/>
     <col min="5" max="5" width="50" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5555555555556" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="7" max="16384" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8485,7 +8676,7 @@
       <c r="B8" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>108</v>
       </c>
       <c r="D8" s="1" t="s">

</xml_diff>